<commit_message>
Improve existing free resources with verified attendance dates, printable PDFs and order formulas
</commit_message>
<xml_diff>
--- a/assets/downloads/homeschool-attendance-sheet.xlsx
+++ b/assets/downloads/homeschool-attendance-sheet.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="1" r:id="Rada014274bd34848"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="1" r:id="R4e65d1e6babb4e63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
         <x:color rgb="FF8A3322"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE2D9"/>
         </x:patternFill>
       </x:fill>
@@ -475,8 +475,8 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
-      <x:c r="A12" s="11" t="d">
-        <x:v>2026-09-08T00:00:00.000Z</x:v>
+      <x:c r="A12" s="11" t="n">
+        <x:v>46273</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
         <x:v>Child A</x:v>
@@ -499,8 +499,8 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
-      <x:c r="A13" s="11" t="d">
-        <x:v>2026-09-08T00:00:00.000Z</x:v>
+      <x:c r="A13" s="11" t="n">
+        <x:v>46273</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
         <x:v>Child B</x:v>
@@ -523,8 +523,8 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
-      <x:c r="A14" s="11" t="d">
-        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      <x:c r="A14" s="11" t="n">
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
         <x:v>Child A</x:v>
@@ -547,8 +547,8 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
-      <x:c r="A15" s="11" t="d">
-        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      <x:c r="A15" s="11" t="n">
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
         <x:v>Child B</x:v>

</xml_diff>

<commit_message>
Improve existing free resources with verified attendance dates, printable PDFs and order formulas (#189)
</commit_message>
<xml_diff>
--- a/assets/downloads/homeschool-attendance-sheet.xlsx
+++ b/assets/downloads/homeschool-attendance-sheet.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="1" r:id="Rada014274bd34848"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="1" r:id="R4e65d1e6babb4e63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -116,7 +116,7 @@
         <x:color rgb="FF8A3322"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE2D9"/>
         </x:patternFill>
       </x:fill>
@@ -475,8 +475,8 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
-      <x:c r="A12" s="11" t="d">
-        <x:v>2026-09-08T00:00:00.000Z</x:v>
+      <x:c r="A12" s="11" t="n">
+        <x:v>46273</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
         <x:v>Child A</x:v>
@@ -499,8 +499,8 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
-      <x:c r="A13" s="11" t="d">
-        <x:v>2026-09-08T00:00:00.000Z</x:v>
+      <x:c r="A13" s="11" t="n">
+        <x:v>46273</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
         <x:v>Child B</x:v>
@@ -523,8 +523,8 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
-      <x:c r="A14" s="11" t="d">
-        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      <x:c r="A14" s="11" t="n">
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
         <x:v>Child A</x:v>
@@ -547,8 +547,8 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
-      <x:c r="A15" s="11" t="d">
-        <x:v>2026-09-09T00:00:00.000Z</x:v>
+      <x:c r="A15" s="11" t="n">
+        <x:v>46274</x:v>
       </x:c>
       <x:c r="B15" s="10" t="str">
         <x:v>Child B</x:v>

</xml_diff>